<commit_message>
Add number and role
</commit_message>
<xml_diff>
--- a/HRManagementAPI/uploads/uploadfile.xlsx
+++ b/HRManagementAPI/uploads/uploadfile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simbe\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7310A6-4709-43B3-93BC-706DBEB53430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF7814B-E04E-4083-B4DC-75DBC2A3F65C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{D637D0AC-18DE-4DD5-9F55-DFCA20DCFFAF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
   <si>
     <t>Last Name</t>
   </si>
@@ -161,13 +161,25 @@
     <t>Health,Dental,Vision</t>
   </si>
   <si>
-    <t>simt1e@tpa.org</t>
-  </si>
-  <si>
-    <t>simt2e@tpa.org</t>
-  </si>
-  <si>
-    <t>simt3we@tpa.org</t>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Phone Number</t>
+  </si>
+  <si>
+    <t>simt1ghe@tpa.org</t>
+  </si>
+  <si>
+    <t>simt2nje@tpa.org</t>
+  </si>
+  <si>
+    <t>simt3whjce@tpa.org</t>
   </si>
 </sst>
 </file>
@@ -245,9 +257,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9E8875A0-54AC-4674-A0C2-8BA507F0DED6}" name="Table1" displayName="Table1" ref="A1:P4" totalsRowShown="0">
-  <autoFilter ref="A1:P4" xr:uid="{9E8875A0-54AC-4674-A0C2-8BA507F0DED6}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9E8875A0-54AC-4674-A0C2-8BA507F0DED6}" name="Table1" displayName="Table1" ref="A1:R4" totalsRowShown="0">
+  <autoFilter ref="A1:R4" xr:uid="{9E8875A0-54AC-4674-A0C2-8BA507F0DED6}"/>
+  <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{92143FC5-C6EF-419E-9DAE-AE42A9697862}" name="Last Name"/>
     <tableColumn id="2" xr3:uid="{76E35C1E-743B-493B-AF83-0EB147353B0E}" name="First Name"/>
     <tableColumn id="3" xr3:uid="{5AF3563C-061C-464F-90C3-A68B0C819253}" name="Date of Hire"/>
@@ -264,6 +276,8 @@
     <tableColumn id="23" xr3:uid="{BC19F106-19A0-4943-BAEE-AEE33090A60F}" name="PTO Tracker"/>
     <tableColumn id="12" xr3:uid="{0CBEEB93-D3B0-48E4-90AB-043F4284A9A8}" name="DL Expiration"/>
     <tableColumn id="13" xr3:uid="{CFDA8DA2-667B-4D64-8512-DA6E53B1493A}" name="Nursing License Expiration"/>
+    <tableColumn id="14" xr3:uid="{62091F86-E439-4291-80E6-D03E81EDF416}" name="Role"/>
+    <tableColumn id="15" xr3:uid="{FA1E2372-FD33-4157-8CA8-23C67751B664}" name="Phone Number"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -586,7 +600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88A21171-38B6-4BF8-8161-BA4A46C2F46F}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.81640625" customWidth="1"/>
@@ -604,9 +618,10 @@
     <col min="14" max="14" width="45.36328125" customWidth="1"/>
     <col min="15" max="15" width="15.1796875" customWidth="1"/>
     <col min="16" max="16" width="27.6328125" customWidth="1"/>
+    <col min="18" max="18" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -655,8 +670,14 @@
       <c r="P1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q1" t="s">
+        <v>41</v>
+      </c>
+      <c r="R1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -673,7 +694,7 @@
         <v>27</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="G2" t="s">
         <v>30</v>
@@ -705,8 +726,14 @@
       <c r="P2" s="2">
         <v>46054</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R2">
+        <v>9296025125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -723,7 +750,7 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
         <v>31</v>
@@ -755,8 +782,14 @@
       <c r="P3" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q3" t="s">
+        <v>43</v>
+      </c>
+      <c r="R3">
+        <v>9236025125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -773,7 +806,7 @@
         <v>29</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G4" t="s">
         <v>32</v>
@@ -805,8 +838,14 @@
       <c r="P4" s="2">
         <v>46045</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+      <c r="R4">
+        <v>9246025125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
@@ -814,7 +853,7 @@
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -823,7 +862,7 @@
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -832,7 +871,7 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -841,14 +880,14 @@
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
@@ -857,7 +896,7 @@
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
@@ -866,7 +905,7 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>

</xml_diff>